<commit_message>
generate all scripts and metrics and disable table normalization
</commit_message>
<xml_diff>
--- a/data/processed/sakila/metrics/combined_generation_query.xlsx
+++ b/data/processed/sakila/metrics/combined_generation_query.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,7 +509,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>gpt5</t>
+          <t>gemini-3-1-flash-lite</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -523,13 +523,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -551,13 +551,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -571,29 +571,21 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n"/>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>mini</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>inline</t>
-        </is>
-      </c>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>business</t>
+          <t>technical</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -608,60 +600,52 @@
     <row r="5">
       <c r="A5" s="1" t="n"/>
       <c r="B5" s="1" t="n"/>
-      <c r="C5" s="1" t="n"/>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>yaml</t>
+        </is>
+      </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
           <t>short</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>gpt5</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>inline</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>business</t>
-        </is>
-      </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -670,7 +654,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -679,17 +663,17 @@
       <c r="C7" s="1" t="n"/>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>technical</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -698,14 +682,14 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n"/>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>mini</t>
+          <t>gpt-5-4-nano</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -719,22 +703,22 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -747,13 +731,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -762,44 +746,32 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>gpt5</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>inline</t>
-        </is>
-      </c>
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="n"/>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>business</t>
+          <t>technical</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -808,56 +780,52 @@
     <row r="11">
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="1" t="n"/>
-      <c r="C11" s="1" t="n"/>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>yaml</t>
+        </is>
+      </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>business</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>mini</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>inline</t>
-        </is>
-      </c>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="n"/>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>business</t>
+          <t>short</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -866,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -875,45 +843,779 @@
       <c r="C13" s="1" t="n"/>
       <c r="D13" s="1" t="inlineStr">
         <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>38</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>gemini-3-1-flash-lite</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>inline</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>10</v>
+      </c>
+      <c r="F14" t="n">
+        <v>17</v>
+      </c>
+      <c r="G14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="1" t="n"/>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
           <t>short</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
+      <c r="E15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" t="n">
+        <v>19</v>
+      </c>
+      <c r="G15" t="n">
+        <v>7</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="1" t="n"/>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>12</v>
+      </c>
+      <c r="F16" t="n">
+        <v>17</v>
+      </c>
+      <c r="G16" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="1" t="n"/>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>yaml</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F17" t="n">
+        <v>18</v>
+      </c>
+      <c r="G17" t="n">
+        <v>7</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="1" t="n"/>
+      <c r="C18" s="1" t="n"/>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>11</v>
+      </c>
+      <c r="F18" t="n">
+        <v>17</v>
+      </c>
+      <c r="G18" t="n">
+        <v>8</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="1" t="n"/>
+      <c r="C19" s="1" t="n"/>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" t="n">
+        <v>18</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n"/>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>gpt-5-4-nano</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>inline</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" t="n">
+        <v>18</v>
+      </c>
+      <c r="G20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n"/>
+      <c r="B21" s="1" t="n"/>
+      <c r="C21" s="1" t="n"/>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" t="n">
+        <v>16</v>
+      </c>
+      <c r="G21" t="n">
+        <v>6</v>
+      </c>
+      <c r="H21" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="1" t="n"/>
+      <c r="C22" s="1" t="n"/>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" t="n">
+        <v>18</v>
+      </c>
+      <c r="G22" t="n">
+        <v>6</v>
+      </c>
+      <c r="H22" t="n">
+        <v>3</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n"/>
+      <c r="B23" s="1" t="n"/>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>yaml</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>8</v>
+      </c>
+      <c r="F23" t="n">
+        <v>18</v>
+      </c>
+      <c r="G23" t="n">
+        <v>6</v>
+      </c>
+      <c r="H23" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n"/>
+      <c r="B24" s="1" t="n"/>
+      <c r="C24" s="1" t="n"/>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>10</v>
+      </c>
+      <c r="F24" t="n">
+        <v>17</v>
+      </c>
+      <c r="G24" t="n">
+        <v>6</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n"/>
+      <c r="B25" s="1" t="n"/>
+      <c r="C25" s="1" t="n"/>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" t="n">
+        <v>19</v>
+      </c>
+      <c r="G25" t="n">
+        <v>8</v>
+      </c>
+      <c r="H25" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>gemini-3-1-flash-lite</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>inline</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>12</v>
+      </c>
+      <c r="J26" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n"/>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="n"/>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>4</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>11</v>
+      </c>
+      <c r="J27" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n"/>
+      <c r="B28" s="1" t="n"/>
+      <c r="C28" s="1" t="n"/>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="n">
+        <v>2</v>
+      </c>
+      <c r="I28" t="n">
+        <v>14</v>
+      </c>
+      <c r="J28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n"/>
+      <c r="B29" s="1" t="n"/>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>yaml</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="n">
+        <v>15</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n"/>
+      <c r="B30" s="1" t="n"/>
+      <c r="C30" s="1" t="n"/>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" t="n">
+        <v>12</v>
+      </c>
+      <c r="J30" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n"/>
+      <c r="B31" s="1" t="n"/>
+      <c r="C31" s="1" t="n"/>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" t="n">
+        <v>12</v>
+      </c>
+      <c r="J31" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n"/>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>gpt-5-4-nano</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>inline</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" t="n">
+        <v>6</v>
+      </c>
+      <c r="J32" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="1" t="n"/>
+      <c r="C33" s="1" t="n"/>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="n">
+        <v>2</v>
+      </c>
+      <c r="I33" t="n">
+        <v>6</v>
+      </c>
+      <c r="J33" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n"/>
+      <c r="B34" s="1" t="n"/>
+      <c r="C34" s="1" t="n"/>
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="n">
+        <v>8</v>
+      </c>
+      <c r="J34" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n"/>
+      <c r="B35" s="1" t="n"/>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>yaml</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="n">
+        <v>8</v>
+      </c>
+      <c r="J35" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n"/>
+      <c r="B36" s="1" t="n"/>
+      <c r="C36" s="1" t="n"/>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3</v>
+      </c>
+      <c r="I36" t="n">
+        <v>4</v>
+      </c>
+      <c r="J36" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="n"/>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" t="n">
+        <v>2</v>
+      </c>
+      <c r="I37" t="n">
+        <v>7</v>
+      </c>
+      <c r="J37" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A10:A13"/>
+  <mergeCells count="21">
+    <mergeCell ref="B32:B37"/>
+    <mergeCell ref="A26:A37"/>
+    <mergeCell ref="A2:A13"/>
+    <mergeCell ref="B26:B31"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="A14:A25"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="B8:B13"/>
+    <mergeCell ref="B2:B7"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="B20:B25"/>
+    <mergeCell ref="C8:C10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>